<commit_message>
only section of dukha remaining bajrayogini valuation given
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/नगर बजेट estimate/छापभन्ज्याङ बज्रयोगिनी मन्दिर पूर्वाधार विकास/छापभन्ज्याङ बज्रयोगिनी मन्दिर पूर्वाधार विकास - Copy.xlsx
+++ b/बजेट माग estimate/नगर बजेट estimate/छापभन्ज्याङ बज्रयोगिनी मन्दिर पूर्वाधार विकास/छापभन्ज्याङ बज्रयोगिनी मन्दिर पूर्वाधार विकास - Copy.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38209D7A-A458-417B-9648-1AF8BF8B9F45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{264BB731-F9E4-4780-B167-C601110DF006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="estimate" sheetId="12" r:id="rId1"/>
@@ -95,7 +95,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="69">
   <si>
     <t>Government of Nepal</t>
   </si>
@@ -256,9 +256,6 @@
     <t xml:space="preserve">F.Y:2082/2083            </t>
   </si>
   <si>
-    <t xml:space="preserve">Date:2082/12/09       </t>
-  </si>
-  <si>
     <t>S.No.</t>
   </si>
   <si>
@@ -308,6 +305,12 @@
   </si>
   <si>
     <t>water</t>
+  </si>
+  <si>
+    <t>Date:2083/02/12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date:2083/02/12       </t>
   </si>
 </sst>
 </file>
@@ -691,10 +694,48 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="43" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -730,45 +771,7 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1574,113 +1577,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="76"/>
+      <c r="I1" s="76"/>
+      <c r="J1" s="76"/>
+      <c r="K1" s="76"/>
     </row>
     <row r="2" spans="1:19" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="65"/>
+      <c r="A2" s="77" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
+      <c r="I2" s="77"/>
+      <c r="J2" s="77"/>
+      <c r="K2" s="77"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" s="66" t="s">
+      <c r="A3" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="66"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
-      <c r="I3" s="66"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="66"/>
+      <c r="B3" s="78"/>
+      <c r="C3" s="78"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="78"/>
+      <c r="F3" s="78"/>
+      <c r="G3" s="78"/>
+      <c r="H3" s="78"/>
+      <c r="I3" s="78"/>
+      <c r="J3" s="78"/>
+      <c r="K3" s="78"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="66"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="66"/>
-      <c r="F4" s="66"/>
-      <c r="G4" s="66"/>
-      <c r="H4" s="66"/>
-      <c r="I4" s="66"/>
-      <c r="J4" s="66"/>
-      <c r="K4" s="66"/>
+      <c r="B4" s="78"/>
+      <c r="C4" s="78"/>
+      <c r="D4" s="78"/>
+      <c r="E4" s="78"/>
+      <c r="F4" s="78"/>
+      <c r="G4" s="78"/>
+      <c r="H4" s="78"/>
+      <c r="I4" s="78"/>
+      <c r="J4" s="78"/>
+      <c r="K4" s="78"/>
     </row>
     <row r="5" spans="1:19" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="67" t="s">
+      <c r="A5" s="79" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="67"/>
-      <c r="C5" s="67"/>
-      <c r="D5" s="67"/>
-      <c r="E5" s="67"/>
-      <c r="F5" s="67"/>
-      <c r="G5" s="67"/>
-      <c r="H5" s="67"/>
-      <c r="I5" s="67"/>
-      <c r="J5" s="67"/>
-      <c r="K5" s="67"/>
+      <c r="B5" s="79"/>
+      <c r="C5" s="79"/>
+      <c r="D5" s="79"/>
+      <c r="E5" s="79"/>
+      <c r="F5" s="79"/>
+      <c r="G5" s="79"/>
+      <c r="H5" s="79"/>
+      <c r="I5" s="79"/>
+      <c r="J5" s="79"/>
+      <c r="K5" s="79"/>
     </row>
     <row r="6" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="62" t="s">
+      <c r="A6" s="66" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="62"/>
-      <c r="C6" s="62"/>
-      <c r="D6" s="62"/>
-      <c r="E6" s="62"/>
-      <c r="F6" s="62"/>
+      <c r="B6" s="66"/>
+      <c r="C6" s="66"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="63" t="s">
+      <c r="H6" s="75" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="63"/>
-      <c r="J6" s="63"/>
-      <c r="K6" s="63"/>
+      <c r="I6" s="75"/>
+      <c r="J6" s="75"/>
+      <c r="K6" s="75"/>
     </row>
     <row r="7" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="70" t="s">
+      <c r="A7" s="82" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="70"/>
-      <c r="C7" s="70"/>
-      <c r="D7" s="70"/>
-      <c r="E7" s="70"/>
-      <c r="F7" s="70"/>
+      <c r="B7" s="82"/>
+      <c r="C7" s="82"/>
+      <c r="D7" s="82"/>
+      <c r="E7" s="82"/>
+      <c r="F7" s="82"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="71" t="s">
+      <c r="H7" s="83" t="s">
         <v>23</v>
       </c>
-      <c r="I7" s="71"/>
-      <c r="J7" s="71"/>
-      <c r="K7" s="71"/>
+      <c r="I7" s="83"/>
+      <c r="J7" s="83"/>
+      <c r="K7" s="83"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
@@ -2847,11 +2850,11 @@
       <c r="B55" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C55" s="68">
+      <c r="C55" s="80">
         <f>J53</f>
         <v>692271.9516078874</v>
       </c>
-      <c r="D55" s="69"/>
+      <c r="D55" s="81"/>
       <c r="E55" s="9">
         <v>100</v>
       </c>
@@ -2873,21 +2876,21 @@
       <c r="B56" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C56" s="72">
+      <c r="C56" s="84">
         <v>600000</v>
       </c>
-      <c r="D56" s="73"/>
+      <c r="D56" s="85"/>
       <c r="E56" s="9"/>
     </row>
     <row r="57" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B57" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C57" s="72">
+      <c r="C57" s="84">
         <f>C56-C59-C60</f>
         <v>570000</v>
       </c>
-      <c r="D57" s="73"/>
+      <c r="D57" s="85"/>
       <c r="E57" s="9">
         <f>C57/C55*100</f>
         <v>82.337584048595986</v>
@@ -2897,11 +2900,11 @@
       <c r="B58" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C58" s="74">
+      <c r="C58" s="86">
         <f>C55-C57</f>
         <v>122271.9516078874</v>
       </c>
-      <c r="D58" s="74"/>
+      <c r="D58" s="86"/>
       <c r="E58" s="9">
         <f>100-E57</f>
         <v>17.662415951404014</v>
@@ -2911,11 +2914,11 @@
       <c r="B59" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C59" s="68">
+      <c r="C59" s="80">
         <f>C56*0.03</f>
         <v>18000</v>
       </c>
-      <c r="D59" s="69"/>
+      <c r="D59" s="81"/>
       <c r="E59" s="9">
         <v>3</v>
       </c>
@@ -2924,24 +2927,17 @@
       <c r="B60" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="C60" s="68">
+      <c r="C60" s="80">
         <f>C56*0.02</f>
         <v>12000</v>
       </c>
-      <c r="D60" s="69"/>
+      <c r="D60" s="81"/>
       <c r="E60" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C59:D59"/>
     <mergeCell ref="C60:D60"/>
     <mergeCell ref="A7:F7"/>
@@ -2950,6 +2946,13 @@
     <mergeCell ref="C56:D56"/>
     <mergeCell ref="C57:D57"/>
     <mergeCell ref="C58:D58"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
@@ -2983,113 +2986,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="76"/>
+      <c r="I1" s="76"/>
+      <c r="J1" s="76"/>
+      <c r="K1" s="76"/>
     </row>
     <row r="2" spans="1:19" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="65"/>
+      <c r="A2" s="77" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
+      <c r="I2" s="77"/>
+      <c r="J2" s="77"/>
+      <c r="K2" s="77"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" s="66" t="s">
+      <c r="A3" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="66"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
-      <c r="I3" s="66"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="66"/>
+      <c r="B3" s="78"/>
+      <c r="C3" s="78"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="78"/>
+      <c r="F3" s="78"/>
+      <c r="G3" s="78"/>
+      <c r="H3" s="78"/>
+      <c r="I3" s="78"/>
+      <c r="J3" s="78"/>
+      <c r="K3" s="78"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="66"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="66"/>
-      <c r="F4" s="66"/>
-      <c r="G4" s="66"/>
-      <c r="H4" s="66"/>
-      <c r="I4" s="66"/>
-      <c r="J4" s="66"/>
-      <c r="K4" s="66"/>
+      <c r="B4" s="78"/>
+      <c r="C4" s="78"/>
+      <c r="D4" s="78"/>
+      <c r="E4" s="78"/>
+      <c r="F4" s="78"/>
+      <c r="G4" s="78"/>
+      <c r="H4" s="78"/>
+      <c r="I4" s="78"/>
+      <c r="J4" s="78"/>
+      <c r="K4" s="78"/>
     </row>
     <row r="5" spans="1:19" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="67" t="s">
+      <c r="A5" s="79" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="67"/>
-      <c r="C5" s="67"/>
-      <c r="D5" s="67"/>
-      <c r="E5" s="67"/>
-      <c r="F5" s="67"/>
-      <c r="G5" s="67"/>
-      <c r="H5" s="67"/>
-      <c r="I5" s="67"/>
-      <c r="J5" s="67"/>
-      <c r="K5" s="67"/>
+      <c r="B5" s="79"/>
+      <c r="C5" s="79"/>
+      <c r="D5" s="79"/>
+      <c r="E5" s="79"/>
+      <c r="F5" s="79"/>
+      <c r="G5" s="79"/>
+      <c r="H5" s="79"/>
+      <c r="I5" s="79"/>
+      <c r="J5" s="79"/>
+      <c r="K5" s="79"/>
     </row>
     <row r="6" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="62" t="s">
+      <c r="A6" s="66" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="62"/>
-      <c r="C6" s="62"/>
-      <c r="D6" s="62"/>
-      <c r="E6" s="62"/>
-      <c r="F6" s="62"/>
+      <c r="B6" s="66"/>
+      <c r="C6" s="66"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="63" t="s">
+      <c r="H6" s="75" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="63"/>
-      <c r="J6" s="63"/>
-      <c r="K6" s="63"/>
+      <c r="I6" s="75"/>
+      <c r="J6" s="75"/>
+      <c r="K6" s="75"/>
     </row>
     <row r="7" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="70" t="s">
+      <c r="A7" s="82" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="70"/>
-      <c r="C7" s="70"/>
-      <c r="D7" s="70"/>
-      <c r="E7" s="70"/>
-      <c r="F7" s="70"/>
+      <c r="B7" s="82"/>
+      <c r="C7" s="82"/>
+      <c r="D7" s="82"/>
+      <c r="E7" s="82"/>
+      <c r="F7" s="82"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="71" t="s">
+      <c r="H7" s="83" t="s">
         <v>23</v>
       </c>
-      <c r="I7" s="71"/>
-      <c r="J7" s="71"/>
-      <c r="K7" s="71"/>
+      <c r="I7" s="83"/>
+      <c r="J7" s="83"/>
+      <c r="K7" s="83"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
@@ -4256,11 +4259,11 @@
       <c r="B55" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C55" s="68">
+      <c r="C55" s="80">
         <f>J53</f>
         <v>692271.9516078874</v>
       </c>
-      <c r="D55" s="69"/>
+      <c r="D55" s="81"/>
       <c r="E55" s="9">
         <v>100</v>
       </c>
@@ -4282,21 +4285,21 @@
       <c r="B56" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C56" s="72">
+      <c r="C56" s="84">
         <v>600000</v>
       </c>
-      <c r="D56" s="73"/>
+      <c r="D56" s="85"/>
       <c r="E56" s="9"/>
     </row>
     <row r="57" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B57" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C57" s="72">
+      <c r="C57" s="84">
         <f>C56-C59-C60</f>
         <v>570000</v>
       </c>
-      <c r="D57" s="73"/>
+      <c r="D57" s="85"/>
       <c r="E57" s="9">
         <f>C57/C55*100</f>
         <v>82.337584048595986</v>
@@ -4306,11 +4309,11 @@
       <c r="B58" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C58" s="74">
+      <c r="C58" s="86">
         <f>C55-C57</f>
         <v>122271.9516078874</v>
       </c>
-      <c r="D58" s="74"/>
+      <c r="D58" s="86"/>
       <c r="E58" s="9">
         <f>100-E57</f>
         <v>17.662415951404014</v>
@@ -4320,11 +4323,11 @@
       <c r="B59" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C59" s="68">
+      <c r="C59" s="80">
         <f>C56*0.03</f>
         <v>18000</v>
       </c>
-      <c r="D59" s="69"/>
+      <c r="D59" s="81"/>
       <c r="E59" s="9">
         <v>3</v>
       </c>
@@ -4333,24 +4336,17 @@
       <c r="B60" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="C60" s="68">
+      <c r="C60" s="80">
         <f>C56*0.02</f>
         <v>12000</v>
       </c>
-      <c r="D60" s="69"/>
+      <c r="D60" s="81"/>
       <c r="E60" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C59:D59"/>
     <mergeCell ref="C60:D60"/>
     <mergeCell ref="A7:F7"/>
@@ -4359,6 +4355,13 @@
     <mergeCell ref="C56:D56"/>
     <mergeCell ref="C57:D57"/>
     <mergeCell ref="C58:D58"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
@@ -4391,90 +4394,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="71" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="77"/>
-      <c r="C1" s="77"/>
-      <c r="D1" s="77"/>
-      <c r="E1" s="77"/>
-      <c r="F1" s="77"/>
-      <c r="G1" s="77"/>
-      <c r="H1" s="77"/>
-      <c r="I1" s="77"/>
-      <c r="J1" s="77"/>
-      <c r="K1" s="77"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
     </row>
     <row r="2" spans="1:13" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="78" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="78"/>
-      <c r="C2" s="78"/>
-      <c r="D2" s="78"/>
-      <c r="E2" s="78"/>
-      <c r="F2" s="78"/>
-      <c r="G2" s="78"/>
-      <c r="H2" s="78"/>
-      <c r="I2" s="78"/>
-      <c r="J2" s="78"/>
-      <c r="K2" s="78"/>
+      <c r="A2" s="72" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
+      <c r="H2" s="72"/>
+      <c r="I2" s="72"/>
+      <c r="J2" s="72"/>
+      <c r="K2" s="72"/>
     </row>
     <row r="3" spans="1:13" s="40" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="79" t="s">
+      <c r="A3" s="73" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="79"/>
-      <c r="C3" s="79"/>
-      <c r="D3" s="79"/>
-      <c r="E3" s="79"/>
-      <c r="F3" s="79"/>
-      <c r="G3" s="79"/>
-      <c r="H3" s="79"/>
-      <c r="I3" s="79"/>
-      <c r="J3" s="79"/>
-      <c r="K3" s="79"/>
+      <c r="B3" s="73"/>
+      <c r="C3" s="73"/>
+      <c r="D3" s="73"/>
+      <c r="E3" s="73"/>
+      <c r="F3" s="73"/>
+      <c r="G3" s="73"/>
+      <c r="H3" s="73"/>
+      <c r="I3" s="73"/>
+      <c r="J3" s="73"/>
+      <c r="K3" s="73"/>
     </row>
     <row r="4" spans="1:13" s="40" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="79" t="s">
+      <c r="A4" s="73" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="79"/>
-      <c r="C4" s="79"/>
-      <c r="D4" s="79"/>
-      <c r="E4" s="79"/>
-      <c r="F4" s="79"/>
-      <c r="G4" s="79"/>
-      <c r="H4" s="79"/>
-      <c r="I4" s="79"/>
-      <c r="J4" s="79"/>
-      <c r="K4" s="79"/>
+      <c r="B4" s="73"/>
+      <c r="C4" s="73"/>
+      <c r="D4" s="73"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="73"/>
+      <c r="H4" s="73"/>
+      <c r="I4" s="73"/>
+      <c r="J4" s="73"/>
+      <c r="K4" s="73"/>
     </row>
     <row r="5" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="80" t="s">
+      <c r="A5" s="74" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="80"/>
-      <c r="C5" s="80"/>
-      <c r="D5" s="80"/>
-      <c r="E5" s="80"/>
-      <c r="F5" s="80"/>
-      <c r="G5" s="80"/>
-      <c r="H5" s="80"/>
-      <c r="I5" s="80"/>
-      <c r="J5" s="80"/>
-      <c r="K5" s="80"/>
+      <c r="B5" s="74"/>
+      <c r="C5" s="74"/>
+      <c r="D5" s="74"/>
+      <c r="E5" s="74"/>
+      <c r="F5" s="74"/>
+      <c r="G5" s="74"/>
+      <c r="H5" s="74"/>
+      <c r="I5" s="74"/>
+      <c r="J5" s="74"/>
+      <c r="K5" s="74"/>
     </row>
     <row r="6" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="41" t="s">
         <v>45</v>
       </c>
       <c r="B6" s="41"/>
-      <c r="C6" s="75">
+      <c r="C6" s="69">
         <f>F34</f>
         <v>692271.9516078874</v>
       </c>
-      <c r="D6" s="76"/>
+      <c r="D6" s="70"/>
       <c r="E6" s="42"/>
       <c r="F6" s="41"/>
       <c r="G6" s="41"/>
@@ -4482,11 +4485,11 @@
         <v>46</v>
       </c>
       <c r="I6" s="41"/>
-      <c r="J6" s="75">
+      <c r="J6" s="69">
         <f>I34</f>
         <v>692428.57611178409</v>
       </c>
-      <c r="K6" s="76"/>
+      <c r="K6" s="70"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="43" t="s">
@@ -4495,78 +4498,78 @@
       <c r="B7" s="43"/>
       <c r="C7" s="43"/>
       <c r="D7" s="43"/>
-      <c r="F7" s="81"/>
-      <c r="G7" s="81"/>
-      <c r="I7" s="82" t="s">
+      <c r="F7" s="64"/>
+      <c r="G7" s="64"/>
+      <c r="I7" s="65" t="s">
         <v>48</v>
       </c>
-      <c r="J7" s="82"/>
-      <c r="K7" s="82"/>
+      <c r="J7" s="65"/>
+      <c r="K7" s="65"/>
     </row>
     <row r="8" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="62" t="s">
+      <c r="A8" s="66" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="62"/>
-      <c r="C8" s="62"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="62"/>
-      <c r="F8" s="62"/>
-      <c r="I8" s="83" t="s">
+      <c r="B8" s="66"/>
+      <c r="C8" s="66"/>
+      <c r="D8" s="66"/>
+      <c r="E8" s="66"/>
+      <c r="F8" s="66"/>
+      <c r="I8" s="67" t="s">
         <v>49</v>
       </c>
-      <c r="J8" s="83"/>
-      <c r="K8" s="83"/>
+      <c r="J8" s="67"/>
+      <c r="K8" s="67"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="84" t="str">
+      <c r="A9" s="68" t="str">
         <f>[7]estimate!A7</f>
         <v>Location:- Shankharapur Municipality 1</v>
       </c>
-      <c r="B9" s="84"/>
-      <c r="C9" s="84"/>
-      <c r="D9" s="84"/>
-      <c r="E9" s="84"/>
-      <c r="F9" s="84"/>
-      <c r="I9" s="83" t="s">
+      <c r="B9" s="68"/>
+      <c r="C9" s="68"/>
+      <c r="D9" s="68"/>
+      <c r="E9" s="68"/>
+      <c r="F9" s="68"/>
+      <c r="I9" s="67" t="s">
+        <v>68</v>
+      </c>
+      <c r="J9" s="67"/>
+      <c r="K9" s="67"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="62" t="s">
         <v>50</v>
       </c>
-      <c r="J9" s="83"/>
-      <c r="K9" s="83"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="86" t="s">
+      <c r="B11" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="86" t="s">
+      <c r="C11" s="62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="63" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="86" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="87" t="s">
+      <c r="E11" s="63"/>
+      <c r="F11" s="63"/>
+      <c r="G11" s="63" t="s">
         <v>53</v>
       </c>
-      <c r="E11" s="87"/>
-      <c r="F11" s="87"/>
-      <c r="G11" s="87" t="s">
+      <c r="H11" s="63"/>
+      <c r="I11" s="63"/>
+      <c r="J11" s="62" t="s">
         <v>54</v>
       </c>
-      <c r="H11" s="87"/>
-      <c r="I11" s="87"/>
-      <c r="J11" s="86" t="s">
+      <c r="K11" s="61" t="s">
         <v>55</v>
       </c>
-      <c r="K11" s="85" t="s">
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="62"/>
+      <c r="B12" s="62"/>
+      <c r="C12" s="62"/>
+      <c r="D12" s="44" t="s">
         <v>56</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="86"/>
-      <c r="B12" s="86"/>
-      <c r="C12" s="86"/>
-      <c r="D12" s="44" t="s">
-        <v>57</v>
       </c>
       <c r="E12" s="44" t="s">
         <v>14</v>
@@ -4575,7 +4578,7 @@
         <v>15</v>
       </c>
       <c r="G12" s="44" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H12" s="44" t="s">
         <v>14</v>
@@ -4583,8 +4586,8 @@
       <c r="I12" s="44" t="s">
         <v>15</v>
       </c>
-      <c r="J12" s="86"/>
-      <c r="K12" s="85"/>
+      <c r="J12" s="62"/>
+      <c r="K12" s="61"/>
     </row>
     <row r="13" spans="1:13" s="40" customFormat="1" ht="126.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="45">
@@ -5191,6 +5194,19 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="I9:K9"/>
     <mergeCell ref="K11:K12"/>
     <mergeCell ref="A11:A12"/>
     <mergeCell ref="B11:B12"/>
@@ -5198,19 +5214,6 @@
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="G11:I11"/>
     <mergeCell ref="J11:J12"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="I7:K7"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5245,113 +5248,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="76"/>
+      <c r="I1" s="76"/>
+      <c r="J1" s="76"/>
+      <c r="K1" s="76"/>
     </row>
     <row r="2" spans="1:16" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="65"/>
+      <c r="A2" s="77" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
+      <c r="I2" s="77"/>
+      <c r="J2" s="77"/>
+      <c r="K2" s="77"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="66" t="s">
+      <c r="A3" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="66"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
-      <c r="I3" s="66"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="66"/>
+      <c r="B3" s="78"/>
+      <c r="C3" s="78"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="78"/>
+      <c r="F3" s="78"/>
+      <c r="G3" s="78"/>
+      <c r="H3" s="78"/>
+      <c r="I3" s="78"/>
+      <c r="J3" s="78"/>
+      <c r="K3" s="78"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="66"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="66"/>
-      <c r="F4" s="66"/>
-      <c r="G4" s="66"/>
-      <c r="H4" s="66"/>
-      <c r="I4" s="66"/>
-      <c r="J4" s="66"/>
-      <c r="K4" s="66"/>
+      <c r="B4" s="78"/>
+      <c r="C4" s="78"/>
+      <c r="D4" s="78"/>
+      <c r="E4" s="78"/>
+      <c r="F4" s="78"/>
+      <c r="G4" s="78"/>
+      <c r="H4" s="78"/>
+      <c r="I4" s="78"/>
+      <c r="J4" s="78"/>
+      <c r="K4" s="78"/>
     </row>
     <row r="5" spans="1:16" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="67" t="s">
-        <v>58</v>
-      </c>
-      <c r="B5" s="67"/>
-      <c r="C5" s="67"/>
-      <c r="D5" s="67"/>
-      <c r="E5" s="67"/>
-      <c r="F5" s="67"/>
-      <c r="G5" s="67"/>
-      <c r="H5" s="67"/>
-      <c r="I5" s="67"/>
-      <c r="J5" s="67"/>
-      <c r="K5" s="67"/>
+      <c r="A5" s="79" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" s="79"/>
+      <c r="C5" s="79"/>
+      <c r="D5" s="79"/>
+      <c r="E5" s="79"/>
+      <c r="F5" s="79"/>
+      <c r="G5" s="79"/>
+      <c r="H5" s="79"/>
+      <c r="I5" s="79"/>
+      <c r="J5" s="79"/>
+      <c r="K5" s="79"/>
     </row>
     <row r="6" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="62" t="s">
+      <c r="A6" s="66" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="62"/>
-      <c r="C6" s="62"/>
-      <c r="D6" s="62"/>
-      <c r="E6" s="62"/>
-      <c r="F6" s="62"/>
+      <c r="B6" s="66"/>
+      <c r="C6" s="66"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="63" t="s">
+      <c r="H6" s="75" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="63"/>
-      <c r="J6" s="63"/>
-      <c r="K6" s="63"/>
+      <c r="I6" s="75"/>
+      <c r="J6" s="75"/>
+      <c r="K6" s="75"/>
     </row>
     <row r="7" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="70" t="s">
+      <c r="A7" s="82" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="70"/>
-      <c r="C7" s="70"/>
-      <c r="D7" s="70"/>
-      <c r="E7" s="70"/>
-      <c r="F7" s="70"/>
+      <c r="B7" s="82"/>
+      <c r="C7" s="82"/>
+      <c r="D7" s="82"/>
+      <c r="E7" s="82"/>
+      <c r="F7" s="82"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="71" t="s">
-        <v>23</v>
-      </c>
-      <c r="I7" s="71"/>
-      <c r="J7" s="71"/>
-      <c r="K7" s="71"/>
+      <c r="H7" s="83" t="s">
+        <v>67</v>
+      </c>
+      <c r="I7" s="83"/>
+      <c r="J7" s="83"/>
+      <c r="K7" s="83"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
@@ -5724,7 +5727,7 @@
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" s="16"/>
       <c r="B21" s="32" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C21" s="17">
         <f t="shared" ref="C21:E23" si="0">C36</f>
@@ -5847,7 +5850,7 @@
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="16"/>
       <c r="B25" s="32" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C25" s="17">
         <v>1</v>
@@ -6141,7 +6144,7 @@
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="16"/>
       <c r="B36" s="32" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C36" s="17">
         <v>1</v>
@@ -6513,7 +6516,7 @@
     <row r="51" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A51" s="16"/>
       <c r="B51" s="32" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C51" s="37">
         <v>1</v>
@@ -6571,7 +6574,7 @@
     <row r="53" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A53" s="16"/>
       <c r="B53" s="32" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C53" s="37">
         <v>1</v>
@@ -6657,7 +6660,7 @@
       <c r="O55" s="36"/>
       <c r="P55" s="36"/>
       <c r="R55" s="19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="S55" s="36">
         <f>J59+J27</f>
@@ -6689,7 +6692,7 @@
       </c>
       <c r="K56" s="5"/>
       <c r="R56" s="19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="S56" s="36">
         <f>J41+J57</f>
@@ -6714,7 +6717,7 @@
       </c>
       <c r="K57" s="17"/>
       <c r="R57" s="19" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="S57" s="36">
         <f>J42+J58</f>
@@ -6739,7 +6742,7 @@
       </c>
       <c r="K58" s="17"/>
       <c r="R58" s="19" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="S58" s="36">
         <f>J60+J45</f>
@@ -6867,13 +6870,13 @@
     <row r="66" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="26"/>
       <c r="B66" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="C66" s="68">
+        <v>58</v>
+      </c>
+      <c r="C66" s="80">
         <f>J64</f>
         <v>692428.57611178409</v>
       </c>
-      <c r="D66" s="69"/>
+      <c r="D66" s="81"/>
       <c r="E66" s="9">
         <v>100</v>
       </c>
@@ -6895,21 +6898,21 @@
       <c r="B67" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C67" s="72">
+      <c r="C67" s="84">
         <v>600000</v>
       </c>
-      <c r="D67" s="73"/>
+      <c r="D67" s="85"/>
       <c r="E67" s="9"/>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B68" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C68" s="72">
+      <c r="C68" s="84">
         <f>C67-C70-C71</f>
         <v>570000</v>
       </c>
-      <c r="D68" s="73"/>
+      <c r="D68" s="85"/>
       <c r="E68" s="9">
         <f>C68/C66*100</f>
         <v>82.318959624794644</v>
@@ -6919,11 +6922,11 @@
       <c r="B69" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C69" s="74">
+      <c r="C69" s="86">
         <f>C66-C68</f>
         <v>122428.57611178409</v>
       </c>
-      <c r="D69" s="74"/>
+      <c r="D69" s="86"/>
       <c r="E69" s="9">
         <f>100-E68</f>
         <v>17.681040375205356</v>
@@ -6933,11 +6936,11 @@
       <c r="B70" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C70" s="68">
+      <c r="C70" s="80">
         <f>C67*0.03</f>
         <v>18000</v>
       </c>
-      <c r="D70" s="69"/>
+      <c r="D70" s="81"/>
       <c r="E70" s="9">
         <v>3</v>
       </c>
@@ -6946,17 +6949,24 @@
       <c r="B71" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="C71" s="68">
+      <c r="C71" s="80">
         <f>C67*0.02</f>
         <v>12000</v>
       </c>
-      <c r="D71" s="69"/>
+      <c r="D71" s="81"/>
       <c r="E71" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C70:D70"/>
     <mergeCell ref="C71:D71"/>
     <mergeCell ref="A7:F7"/>
@@ -6965,22 +6975,12 @@
     <mergeCell ref="C67:D67"/>
     <mergeCell ref="C68:D68"/>
     <mergeCell ref="C69:D69"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
   </headerFooter>
-  <rowBreaks count="1" manualBreakCount="1">
-    <brk id="46" max="10" man="1"/>
-  </rowBreaks>
 </worksheet>
 </file>
 
@@ -7005,110 +7005,110 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="76"/>
+      <c r="I1" s="76"/>
+      <c r="J1" s="76"/>
+      <c r="K1" s="76"/>
     </row>
     <row r="2" spans="1:16" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="65"/>
+      <c r="A2" s="77" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
+      <c r="I2" s="77"/>
+      <c r="J2" s="77"/>
+      <c r="K2" s="77"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="66" t="s">
+      <c r="A3" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="66"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
-      <c r="I3" s="66"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="66"/>
+      <c r="B3" s="78"/>
+      <c r="C3" s="78"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="78"/>
+      <c r="F3" s="78"/>
+      <c r="G3" s="78"/>
+      <c r="H3" s="78"/>
+      <c r="I3" s="78"/>
+      <c r="J3" s="78"/>
+      <c r="K3" s="78"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="66" t="s">
+      <c r="A4" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="66"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="66"/>
-      <c r="F4" s="66"/>
-      <c r="G4" s="66"/>
-      <c r="H4" s="66"/>
-      <c r="I4" s="66"/>
-      <c r="J4" s="66"/>
-      <c r="K4" s="66"/>
+      <c r="B4" s="78"/>
+      <c r="C4" s="78"/>
+      <c r="D4" s="78"/>
+      <c r="E4" s="78"/>
+      <c r="F4" s="78"/>
+      <c r="G4" s="78"/>
+      <c r="H4" s="78"/>
+      <c r="I4" s="78"/>
+      <c r="J4" s="78"/>
+      <c r="K4" s="78"/>
     </row>
     <row r="5" spans="1:16" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="67" t="s">
-        <v>63</v>
-      </c>
-      <c r="B5" s="67"/>
-      <c r="C5" s="67"/>
-      <c r="D5" s="67"/>
-      <c r="E5" s="67"/>
-      <c r="F5" s="67"/>
-      <c r="G5" s="67"/>
-      <c r="H5" s="67"/>
-      <c r="I5" s="67"/>
-      <c r="J5" s="67"/>
-      <c r="K5" s="67"/>
+      <c r="A5" s="79" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="79"/>
+      <c r="C5" s="79"/>
+      <c r="D5" s="79"/>
+      <c r="E5" s="79"/>
+      <c r="F5" s="79"/>
+      <c r="G5" s="79"/>
+      <c r="H5" s="79"/>
+      <c r="I5" s="79"/>
+      <c r="J5" s="79"/>
+      <c r="K5" s="79"/>
     </row>
     <row r="6" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="62" t="s">
+      <c r="A6" s="66" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="62"/>
-      <c r="C6" s="62"/>
-      <c r="D6" s="62"/>
-      <c r="E6" s="62"/>
-      <c r="F6" s="62"/>
+      <c r="B6" s="66"/>
+      <c r="C6" s="66"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
       <c r="G6" s="10"/>
-      <c r="I6" s="61"/>
-      <c r="J6" s="61"/>
+      <c r="I6" s="60"/>
+      <c r="J6" s="60"/>
       <c r="K6" s="39" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="70" t="s">
+      <c r="A7" s="82" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="70"/>
-      <c r="C7" s="70"/>
-      <c r="D7" s="70"/>
-      <c r="E7" s="70"/>
-      <c r="F7" s="70"/>
+      <c r="B7" s="82"/>
+      <c r="C7" s="82"/>
+      <c r="D7" s="82"/>
+      <c r="E7" s="82"/>
+      <c r="F7" s="82"/>
       <c r="G7" s="11"/>
-      <c r="I7" s="60"/>
-      <c r="J7" s="60"/>
+      <c r="I7" s="87"/>
+      <c r="J7" s="87"/>
       <c r="K7" s="38" t="s">
-        <v>23</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
@@ -7482,7 +7482,7 @@
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" s="16"/>
       <c r="B21" s="32" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C21" s="17">
         <f t="shared" ref="C21:E23" si="0">C36</f>
@@ -7605,7 +7605,7 @@
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="16"/>
       <c r="B25" s="32" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C25" s="17">
         <v>1</v>
@@ -7899,7 +7899,7 @@
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" s="16"/>
       <c r="B36" s="32" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C36" s="17">
         <v>1</v>
@@ -8271,7 +8271,7 @@
     <row r="51" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A51" s="16"/>
       <c r="B51" s="32" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C51" s="37">
         <v>1</v>
@@ -8329,7 +8329,7 @@
     <row r="53" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A53" s="16"/>
       <c r="B53" s="32" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C53" s="37">
         <v>1</v>
@@ -8597,13 +8597,13 @@
     <row r="66" spans="1:19" s="20" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="26"/>
       <c r="B66" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="C66" s="68">
+        <v>58</v>
+      </c>
+      <c r="C66" s="80">
         <f>J64</f>
         <v>692428.57611178409</v>
       </c>
-      <c r="D66" s="69"/>
+      <c r="D66" s="81"/>
       <c r="E66" s="9">
         <v>100</v>
       </c>
@@ -8625,21 +8625,21 @@
       <c r="B67" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C67" s="72">
+      <c r="C67" s="84">
         <v>600000</v>
       </c>
-      <c r="D67" s="73"/>
+      <c r="D67" s="85"/>
       <c r="E67" s="9"/>
     </row>
     <row r="68" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="B68" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C68" s="72">
+      <c r="C68" s="84">
         <f>C67-C70-C71</f>
         <v>570000</v>
       </c>
-      <c r="D68" s="73"/>
+      <c r="D68" s="85"/>
       <c r="E68" s="9">
         <f>C68/C66*100</f>
         <v>82.318959624794644</v>
@@ -8649,11 +8649,11 @@
       <c r="B69" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C69" s="74">
+      <c r="C69" s="86">
         <f>C66-C68</f>
         <v>122428.57611178409</v>
       </c>
-      <c r="D69" s="74"/>
+      <c r="D69" s="86"/>
       <c r="E69" s="9">
         <f>100-E68</f>
         <v>17.681040375205356</v>
@@ -8663,11 +8663,11 @@
       <c r="B70" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C70" s="68">
+      <c r="C70" s="80">
         <f>C67*0.03</f>
         <v>18000</v>
       </c>
-      <c r="D70" s="69"/>
+      <c r="D70" s="81"/>
       <c r="E70" s="9">
         <v>3</v>
       </c>
@@ -8676,23 +8676,17 @@
       <c r="B71" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="C71" s="68">
+      <c r="C71" s="80">
         <f>C67*0.02</f>
         <v>12000</v>
       </c>
-      <c r="D71" s="69"/>
+      <c r="D71" s="81"/>
       <c r="E71" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C70:D70"/>
     <mergeCell ref="C71:D71"/>
     <mergeCell ref="A7:F7"/>
@@ -8700,14 +8694,17 @@
     <mergeCell ref="C67:D67"/>
     <mergeCell ref="C68:D68"/>
     <mergeCell ref="C69:D69"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
-  <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="95" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
   </headerFooter>
-  <rowBreaks count="1" manualBreakCount="1">
-    <brk id="46" max="10" man="1"/>
-  </rowBreaks>
 </worksheet>
 </file>
</xml_diff>